<commit_message>
20260512 worked on project, notebook
</commit_message>
<xml_diff>
--- a/chemistry_book/content/project_THe/datasets/df_lab_macros.xlsx
+++ b/chemistry_book/content/project_THe/datasets/df_lab_macros.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="33">
   <si>
     <t>measpointname</t>
   </si>
@@ -101,6 +101,9 @@
   </si>
   <si>
     <t>IDS-put 6</t>
+  </si>
+  <si>
+    <t>Temperatuur</t>
   </si>
   <si>
     <t>PP-11N</t>
@@ -171,8 +174,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:C113" totalsRowShown="0">
-  <autoFilter ref="A1:C113"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:C117" totalsRowShown="0">
+  <autoFilter ref="A1:C117"/>
   <tableColumns count="3">
     <tableColumn id="1" name="measpointname" dataDxfId="0"/>
     <tableColumn id="2" name="cname" dataDxfId="0"/>
@@ -467,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -992,10 +995,10 @@
         <v>28</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C48" s="2">
-        <v>71</v>
+        <v>284</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -1003,10 +1006,10 @@
         <v>28</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C49" s="2">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1014,241 +1017,241 @@
         <v>28</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="C50" s="2">
-        <v>286</v>
+        <v>61</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C51" s="2">
-        <v>68</v>
+        <v>286</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C52" s="2">
-        <v>482</v>
+        <v>68</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C53" s="2">
-        <v>102</v>
+        <v>482</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C54" s="2">
-        <v>276</v>
+        <v>102</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C55" s="2">
-        <v>94</v>
+        <v>276</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C56" s="2">
-        <v>82</v>
+        <v>94</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C57" s="2">
-        <v>314</v>
+        <v>82</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C58" s="2">
-        <v>128</v>
+        <v>314</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C59" s="2">
-        <v>33</v>
+        <v>128</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C60" s="2">
-        <v>44</v>
+        <v>33</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C61" s="2">
-        <v>78</v>
+        <v>44</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C62" s="2">
-        <v>57</v>
+        <v>78</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C63" s="2">
-        <v>72</v>
+        <v>57</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C64" s="2">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C65" s="2">
-        <v>80</v>
+        <v>68</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C66" s="2">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C67" s="2">
-        <v>462</v>
+        <v>69</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C68" s="2">
-        <v>79</v>
+        <v>462</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C69" s="2">
-        <v>62</v>
+        <v>79</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B70" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B70" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="C70" s="2">
-        <v>76</v>
+        <v>285</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="C71" s="2">
-        <v>299</v>
+        <v>62</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -1256,10 +1259,10 @@
         <v>30</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C72" s="2">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -1267,219 +1270,219 @@
         <v>30</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C73" s="2">
-        <v>476</v>
+        <v>299</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C74" s="2">
-        <v>101</v>
+        <v>72</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C75" s="2">
-        <v>255</v>
+        <v>476</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C76" s="2">
-        <v>85</v>
+        <v>101</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C77" s="2">
-        <v>84</v>
+        <v>255</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C78" s="2">
-        <v>316</v>
+        <v>85</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C79" s="2">
-        <v>128</v>
+        <v>84</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C80" s="2">
-        <v>41</v>
+        <v>316</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C81" s="2">
-        <v>52</v>
+        <v>128</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C82" s="2">
-        <v>75</v>
+        <v>41</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C83" s="2">
-        <v>58</v>
+        <v>52</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C84" s="2">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C85" s="2">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C86" s="2">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C87" s="2">
-        <v>70</v>
+        <v>61</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C88" s="2">
-        <v>478</v>
+        <v>79</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C89" s="2">
-        <v>81</v>
+        <v>70</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C90" s="2">
-        <v>59</v>
+        <v>478</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C91" s="2">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="C92" s="2">
-        <v>306</v>
+        <v>293</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -1487,10 +1490,10 @@
         <v>31</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C93" s="2">
-        <v>77</v>
+        <v>59</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -1498,10 +1501,10 @@
         <v>31</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="C94" s="2">
-        <v>450</v>
+        <v>82</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -1509,207 +1512,251 @@
         <v>31</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C95" s="2">
-        <v>103</v>
+        <v>306</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C96" s="2">
-        <v>241</v>
+        <v>77</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C97" s="2">
-        <v>88</v>
+        <v>450</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C98" s="2">
-        <v>88</v>
+        <v>103</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C99" s="2">
-        <v>300</v>
+        <v>241</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C100" s="2">
-        <v>135</v>
+        <v>88</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C101" s="2">
-        <v>46</v>
+        <v>88</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C102" s="2">
-        <v>63</v>
+        <v>300</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C103" s="2">
-        <v>87</v>
+        <v>135</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C104" s="2">
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C105" s="2">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C106" s="2">
-        <v>71</v>
+        <v>87</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C107" s="2">
-        <v>84</v>
+        <v>62</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C108" s="2">
-        <v>65</v>
+        <v>71</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C109" s="2">
-        <v>481</v>
+        <v>71</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C110" s="2">
-        <v>97</v>
+        <v>84</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C111" s="2">
-        <v>58</v>
+        <v>65</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C112" s="2">
-        <v>86</v>
+        <v>481</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B113" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C113" s="2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3">
+      <c r="A114" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C114" s="2">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3">
+      <c r="A115" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C115" s="2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3">
+      <c r="A116" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C116" s="2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3">
+      <c r="A117" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B117" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C113" s="2">
+      <c r="C117" s="2">
         <v>305</v>
       </c>
     </row>

</xml_diff>